<commit_message>
feat: adding new metric and baseline
</commit_message>
<xml_diff>
--- a/results/20250624/evaluation_CHD_49_noisy_0.0_br.xlsx
+++ b/results/20250624/evaluation_CHD_49_noisy_0.0_br.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,14 +573,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>mfrd</t>
+          <t>jaccard</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>0.52222</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>0.01482</v>
       </c>
     </row>
     <row r="6">
@@ -600,13 +600,256 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>macro_f1</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0.47658</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.01721</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BinaryVector</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>micro_f1</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>0.6616300000000001</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.01745</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>BinaryVector</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>macro_precision</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>0.5176500000000001</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.01351</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>BinaryVector</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>micro_precision</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0.66803</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.02025</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>BinaryVector</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>macro_recall</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>0.47939</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.02575</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>BinaryVector</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>micro_recall</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>0.65656</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.03141</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>BinaryVector</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>example_precision</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>0.6776</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.02265</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>BinaryVector</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>example_recall</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>0.64619</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.0313</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>BinaryVector</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>mfrd</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>BinaryVector</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
           <t>afrd</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="H15" t="n">
         <v>0.62602</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I15" t="n">
         <v>0.03869</v>
       </c>
     </row>

</xml_diff>